<commit_message>
Piping package (routing, 13 isometrics, stress study, MTO, piping 3D); full rebuild; README
- P-119 placed in layout and mechanical pump data; multi-bay air coolers placed contiguously
- Clean end-to-end build of all 12 stages

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013qGZUcwwWBAcAEPeh7Toud
</commit_message>
<xml_diff>
--- a/deliverables/02-equipment/CFU-000-ME-DS-000_Equipment-Datasheets-Combined.xlsx
+++ b/deliverables/02-equipment/CFU-000-ME-DS-000_Equipment-Datasheets-Combined.xlsx
@@ -620,7 +620,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>P-101A/B, P-102A/B, P-103A/B, P-104A/B, P-105A/B, P-106A/B, P-107A/B, P-108A/B, P-109A/B, P-110A/B, P-111A/B, P-112A/B, P-114A/B, P-115A/B, P-116A/B, P-117A/B, P-118, P-201A/B, P-202A/B, P-203A/B, P-204A/B, P-205A/B, P-206A/B</t>
+          <t>P-101A/B, P-102A/B, P-103A/B, P-104A/B, P-105A/B, P-106A/B, P-107A/B, P-108A/B, P-109A/B, P-110A/B, P-111A/B, P-112A/B, P-114A/B, P-115A/B, P-116A/B, P-117A/B, P-118, P-119A/B, P-201A/B, P-202A/B, P-203A/B, P-204A/B, P-205A/B, P-206A/B</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PSV-1001, PSV-1002, PSV-1003, PSV-1004, PSV-1005, PSV-1006, PSV-1007, PSV-1008, PSV-1009, PSV-1010, PSV-2001, PSV-2002</t>
+          <t>PSV-1001, PSV-1002, PSV-1003, PSV-1004, PSV-1005, PSV-1006, PSV-1007, PSV-1008, PSV-1009, PSV-1010, PSV-2001, PSV-2002, PSV-1011, PSV-2003, TSV-typ</t>
         </is>
       </c>
     </row>
@@ -14652,57 +14652,57 @@
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>30 / 20 barg</t>
+          <t>35 / 20 barg</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>30 / 20 barg</t>
+          <t>35 / 20 barg</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>30 / 20 barg</t>
+          <t>35 / 20 barg</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
-          <t>30 / 20 barg</t>
+          <t>35 / 20 barg</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>30 / 20 barg</t>
+          <t>35 / 20 barg</t>
         </is>
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>30 / 20 barg</t>
+          <t>45 / 20 barg</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr">
         <is>
-          <t>30 / 20 barg</t>
+          <t>45 / 20 barg</t>
         </is>
       </c>
       <c r="J22" s="10" t="inlineStr">
         <is>
-          <t>30 / 20 barg</t>
+          <t>45 / 20 barg</t>
         </is>
       </c>
       <c r="K22" s="10" t="inlineStr">
         <is>
-          <t>30 / 20 barg</t>
+          <t>45 / 20 barg</t>
         </is>
       </c>
       <c r="L22" s="10" t="inlineStr">
         <is>
-          <t>30 / 20 barg</t>
+          <t>45 / 20 barg</t>
         </is>
       </c>
       <c r="M22" s="10" t="inlineStr">
         <is>
-          <t>30 / 20 barg</t>
+          <t>45 / 20 barg</t>
         </is>
       </c>
       <c r="N22" s="10" t="inlineStr">
@@ -14878,57 +14878,57 @@
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>39.0 / 26.0 barg</t>
+          <t>45.5 / 26.0 barg</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>39.0 / 26.0 barg</t>
+          <t>45.5 / 26.0 barg</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>39.0 / 26.0 barg</t>
+          <t>45.5 / 26.0 barg</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>39.0 / 26.0 barg</t>
+          <t>45.5 / 26.0 barg</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>39.0 / 26.0 barg</t>
+          <t>45.5 / 26.0 barg</t>
         </is>
       </c>
       <c r="H24" s="10" t="inlineStr">
         <is>
-          <t>39.0 / 26.0 barg</t>
+          <t>58.5 / 26.0 barg</t>
         </is>
       </c>
       <c r="I24" s="10" t="inlineStr">
         <is>
-          <t>39.0 / 26.0 barg</t>
+          <t>58.5 / 26.0 barg</t>
         </is>
       </c>
       <c r="J24" s="10" t="inlineStr">
         <is>
-          <t>39.0 / 26.0 barg</t>
+          <t>58.5 / 26.0 barg</t>
         </is>
       </c>
       <c r="K24" s="10" t="inlineStr">
         <is>
-          <t>39.0 / 26.0 barg</t>
+          <t>58.5 / 26.0 barg</t>
         </is>
       </c>
       <c r="L24" s="10" t="inlineStr">
         <is>
-          <t>39.0 / 26.0 barg</t>
+          <t>58.5 / 26.0 barg</t>
         </is>
       </c>
       <c r="M24" s="10" t="inlineStr">
         <is>
-          <t>39.0 / 26.0 barg</t>
+          <t>58.5 / 26.0 barg</t>
         </is>
       </c>
       <c r="N24" s="10" t="inlineStr">
@@ -15242,32 +15242,32 @@
       </c>
       <c r="H27" s="10" t="inlineStr">
         <is>
-          <t>16" 300#</t>
+          <t>16" 600#</t>
         </is>
       </c>
       <c r="I27" s="10" t="inlineStr">
         <is>
-          <t>16" 300#</t>
+          <t>16" 600#</t>
         </is>
       </c>
       <c r="J27" s="10" t="inlineStr">
         <is>
-          <t>16" 300#</t>
+          <t>16" 600#</t>
         </is>
       </c>
       <c r="K27" s="10" t="inlineStr">
         <is>
-          <t>16" 300#</t>
+          <t>16" 600#</t>
         </is>
       </c>
       <c r="L27" s="10" t="inlineStr">
         <is>
-          <t>16" 300#</t>
+          <t>16" 600#</t>
         </is>
       </c>
       <c r="M27" s="10" t="inlineStr">
         <is>
-          <t>8" 300#</t>
+          <t>8" 600#</t>
         </is>
       </c>
       <c r="N27" s="10" t="inlineStr">
@@ -15782,57 +15782,57 @@
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>SA-516-70 / 1200 mm / 20 mm</t>
+          <t>SA-516-70 / 1200 mm / 22 mm</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>SA-516-70 / 1300 mm / 20 mm</t>
+          <t>SA-516-70 / 1300 mm / 25 mm</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr">
         <is>
-          <t>SA-516-70 / 1250 mm / 20 mm</t>
+          <t>SA-516-70 / 1250 mm / 25 mm</t>
         </is>
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
-          <t>SA-516-70 / 1200 mm / 20 mm</t>
+          <t>SA-516-70 / 1200 mm / 22 mm</t>
         </is>
       </c>
       <c r="G32" s="10" t="inlineStr">
         <is>
-          <t>SA-516-70 / 1300 mm / 22 mm</t>
+          <t>SA-516-70 / 1300 mm / 25 mm</t>
         </is>
       </c>
       <c r="H32" s="10" t="inlineStr">
         <is>
-          <t>SA-516-70 / 1350 mm / 22 mm</t>
+          <t>SA-516-70 / 1350 mm / 30 mm</t>
         </is>
       </c>
       <c r="I32" s="10" t="inlineStr">
         <is>
-          <t>SA-516-70 / 1150 mm / 22 mm</t>
+          <t>SA-516-70 / 1150 mm / 30 mm</t>
         </is>
       </c>
       <c r="J32" s="10" t="inlineStr">
         <is>
-          <t>SA-387-11-2 / 1400 mm / 25 mm</t>
+          <t>SA-387-11-2 / 1400 mm / 32 mm</t>
         </is>
       </c>
       <c r="K32" s="10" t="inlineStr">
         <is>
-          <t>SA-387-11-2 / 1000 mm / 20 mm</t>
+          <t>SA-387-11-2 / 1000 mm / 25 mm</t>
         </is>
       </c>
       <c r="L32" s="10" t="inlineStr">
         <is>
-          <t>SA-387-11-2 / 1300 mm / 22 mm</t>
+          <t>SA-387-11-2 / 1300 mm / 32 mm</t>
         </is>
       </c>
       <c r="M32" s="10" t="inlineStr">
         <is>
-          <t>SA-387-11-2 / 1400 mm / 25 mm</t>
+          <t>SA-387-11-2 / 1400 mm / 36 mm</t>
         </is>
       </c>
       <c r="N32" s="10" t="inlineStr">
@@ -16912,57 +16912,57 @@
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>18.9 / 27.2 t</t>
+          <t>19.4 / 27.6 t</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>22.4 / 32.0 t</t>
+          <t>23.6 / 33.3 t</t>
         </is>
       </c>
       <c r="E42" s="10" t="inlineStr">
         <is>
-          <t>20.7 / 29.6 t</t>
+          <t>21.9 / 30.8 t</t>
         </is>
       </c>
       <c r="F42" s="10" t="inlineStr">
         <is>
-          <t>19.5 / 27.7 t</t>
+          <t>20.0 / 28.2 t</t>
         </is>
       </c>
       <c r="G42" s="10" t="inlineStr">
         <is>
-          <t>22.7 / 32.3 t</t>
+          <t>23.4 / 33.1 t</t>
         </is>
       </c>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>25.2 / 35.6 t</t>
+          <t>27.3 / 37.7 t</t>
         </is>
       </c>
       <c r="I42" s="10" t="inlineStr">
         <is>
-          <t>18.2 / 25.8 t</t>
+          <t>20.0 / 27.6 t</t>
         </is>
       </c>
       <c r="J42" s="10" t="inlineStr">
         <is>
-          <t>28.2 / 39.3 t</t>
+          <t>30.1 / 41.2 t</t>
         </is>
       </c>
       <c r="K42" s="10" t="inlineStr">
         <is>
-          <t>14.5 / 20.2 t</t>
+          <t>15.5 / 21.2 t</t>
         </is>
       </c>
       <c r="L42" s="10" t="inlineStr">
         <is>
-          <t>23.2 / 32.9 t</t>
+          <t>25.7 / 35.4 t</t>
         </is>
       </c>
       <c r="M42" s="10" t="inlineStr">
         <is>
-          <t>28.1 / 39.3 t</t>
+          <t>31.1 / 42.3 t</t>
         </is>
       </c>
       <c r="N42" s="10" t="inlineStr">
@@ -19306,7 +19306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y40"/>
+  <dimension ref="A1:Z40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -19334,6 +19334,7 @@
     <col width="22" customWidth="1" min="23" max="23"/>
     <col width="22" customWidth="1" min="24" max="24"/>
     <col width="22" customWidth="1" min="25" max="25"/>
+    <col width="22" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19366,6 +19367,7 @@
       <c r="W1" t="inlineStr"/>
       <c r="X1" t="inlineStr"/>
       <c r="Y1" t="inlineStr"/>
+      <c r="Z1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -19465,30 +19467,35 @@
       </c>
       <c r="T2" s="5" t="inlineStr">
         <is>
+          <t>P-119A/B</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
           <t>P-201A/B</t>
         </is>
       </c>
-      <c r="U2" s="5" t="inlineStr">
+      <c r="V2" s="5" t="inlineStr">
         <is>
           <t>P-202A/B</t>
         </is>
       </c>
-      <c r="V2" s="5" t="inlineStr">
+      <c r="W2" s="5" t="inlineStr">
         <is>
           <t>P-203A/B</t>
         </is>
       </c>
-      <c r="W2" s="5" t="inlineStr">
+      <c r="X2" s="5" t="inlineStr">
         <is>
           <t>P-204A/B</t>
         </is>
       </c>
-      <c r="X2" s="5" t="inlineStr">
+      <c r="Y2" s="5" t="inlineStr">
         <is>
           <t>P-205A/B</t>
         </is>
       </c>
-      <c r="Y2" s="5" t="inlineStr">
+      <c r="Z2" s="5" t="inlineStr">
         <is>
           <t>P-206A/B</t>
         </is>
@@ -19524,6 +19531,7 @@
       <c r="W3" s="8" t="n"/>
       <c r="X3" s="8" t="n"/>
       <c r="Y3" s="8" t="n"/>
+      <c r="Z3" s="8" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr"/>
@@ -19647,6 +19655,11 @@
           <t>API 610 12th ed. / ISO 13709</t>
         </is>
       </c>
+      <c r="Z4" s="10" t="inlineStr">
+        <is>
+          <t>API 610 12th ed. / ISO 13709</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr"/>
@@ -19742,30 +19755,35 @@
       </c>
       <c r="T5" s="10" t="inlineStr">
         <is>
+          <t>OH2</t>
+        </is>
+      </c>
+      <c r="U5" s="10" t="inlineStr">
+        <is>
           <t>BB2</t>
         </is>
       </c>
-      <c r="U5" s="10" t="inlineStr">
+      <c r="V5" s="10" t="inlineStr">
         <is>
           <t>BB2</t>
         </is>
       </c>
-      <c r="V5" s="10" t="inlineStr">
+      <c r="W5" s="10" t="inlineStr">
         <is>
           <t>BB2</t>
         </is>
       </c>
-      <c r="W5" s="10" t="inlineStr">
+      <c r="X5" s="10" t="inlineStr">
         <is>
           <t>BB2</t>
         </is>
       </c>
-      <c r="X5" s="10" t="inlineStr">
+      <c r="Y5" s="10" t="inlineStr">
         <is>
           <t>OH2</t>
         </is>
       </c>
-      <c r="Y5" s="10" t="inlineStr">
+      <c r="Z5" s="10" t="inlineStr">
         <is>
           <t>API 674/675 PD</t>
         </is>
@@ -19893,6 +19911,11 @@
           <t>2 (1 operating + 1 spare)</t>
         </is>
       </c>
+      <c r="Z6" s="10" t="inlineStr">
+        <is>
+          <t>2 (1 operating + 1 spare)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr"/>
@@ -19988,30 +20011,35 @@
       </c>
       <c r="T7" s="10" t="inlineStr">
         <is>
+          <t>Flare KO drum pump-out</t>
+        </is>
+      </c>
+      <c r="U7" s="10" t="inlineStr">
+        <is>
           <t>LVGO pumparound / product</t>
         </is>
       </c>
-      <c r="U7" s="10" t="inlineStr">
+      <c r="V7" s="10" t="inlineStr">
         <is>
           <t>HVGO pumparound / product</t>
         </is>
       </c>
-      <c r="V7" s="10" t="inlineStr">
+      <c r="W7" s="10" t="inlineStr">
         <is>
           <t>Slop wax</t>
         </is>
       </c>
-      <c r="W7" s="10" t="inlineStr">
+      <c r="X7" s="10" t="inlineStr">
         <is>
           <t>Vacuum residue (incl. quench)</t>
         </is>
       </c>
-      <c r="X7" s="10" t="inlineStr">
+      <c r="Y7" s="10" t="inlineStr">
         <is>
           <t>Hotwell sour water</t>
         </is>
       </c>
-      <c r="Y7" s="10" t="inlineStr">
+      <c r="Z7" s="10" t="inlineStr">
         <is>
           <t>Hotwell slop oil</t>
         </is>
@@ -20139,6 +20167,11 @@
           <t>Electric motor</t>
         </is>
       </c>
+      <c r="Z8" s="10" t="inlineStr">
+        <is>
+          <t>Electric motor</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr"/>
@@ -20234,30 +20267,35 @@
       </c>
       <c r="T9" s="10" t="inlineStr">
         <is>
+          <t>D-104 flare KO drum (liquid at bubble point, 0.2 barg)</t>
+        </is>
+      </c>
+      <c r="U9" s="10" t="inlineStr">
+        <is>
           <t>C-201 LVGO collector</t>
         </is>
       </c>
-      <c r="U9" s="10" t="inlineStr">
+      <c r="V9" s="10" t="inlineStr">
         <is>
           <t>C-201 HVGO collector</t>
         </is>
       </c>
-      <c r="V9" s="10" t="inlineStr">
+      <c r="W9" s="10" t="inlineStr">
         <is>
           <t>C-201 slop wax collector</t>
         </is>
       </c>
-      <c r="W9" s="10" t="inlineStr">
+      <c r="X9" s="10" t="inlineStr">
         <is>
           <t>C-201 boot (quenched VR)</t>
         </is>
       </c>
-      <c r="X9" s="10" t="inlineStr">
+      <c r="Y9" s="10" t="inlineStr">
         <is>
           <t>D-201 hotwell water compartment</t>
         </is>
       </c>
-      <c r="Y9" s="10" t="inlineStr">
+      <c r="Z9" s="10" t="inlineStr">
         <is>
           <t>D-201 slop oil compartment</t>
         </is>
@@ -20293,6 +20331,7 @@
       <c r="W10" s="8" t="n"/>
       <c r="X10" s="8" t="n"/>
       <c r="Y10" s="8" t="n"/>
+      <c r="Z10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr"/>
@@ -20388,30 +20427,35 @@
       </c>
       <c r="T11" s="10" t="inlineStr">
         <is>
+          <t>Flare KO drum pump-out</t>
+        </is>
+      </c>
+      <c r="U11" s="10" t="inlineStr">
+        <is>
           <t>LVGO pumparound / product</t>
         </is>
       </c>
-      <c r="U11" s="10" t="inlineStr">
+      <c r="V11" s="10" t="inlineStr">
         <is>
           <t>HVGO pumparound / product</t>
         </is>
       </c>
-      <c r="V11" s="10" t="inlineStr">
+      <c r="W11" s="10" t="inlineStr">
         <is>
           <t>Slop wax</t>
         </is>
       </c>
-      <c r="W11" s="10" t="inlineStr">
+      <c r="X11" s="10" t="inlineStr">
         <is>
           <t>Vacuum residue (incl. quench)</t>
         </is>
       </c>
-      <c r="X11" s="10" t="inlineStr">
+      <c r="Y11" s="10" t="inlineStr">
         <is>
           <t>Hotwell sour water</t>
         </is>
       </c>
-      <c r="Y11" s="10" t="inlineStr">
+      <c r="Z11" s="10" t="inlineStr">
         <is>
           <t>Hotwell slop oil</t>
         </is>
@@ -20511,30 +20555,35 @@
       </c>
       <c r="T12" s="10" t="inlineStr">
         <is>
+          <t>60 / 90 C</t>
+        </is>
+      </c>
+      <c r="U12" s="10" t="inlineStr">
+        <is>
           <t>224 / 255 C</t>
         </is>
       </c>
-      <c r="U12" s="10" t="inlineStr">
+      <c r="V12" s="10" t="inlineStr">
         <is>
           <t>315 / 345 C</t>
         </is>
       </c>
-      <c r="V12" s="10" t="inlineStr">
+      <c r="W12" s="10" t="inlineStr">
         <is>
           <t>378 / 410 C</t>
         </is>
       </c>
-      <c r="W12" s="10" t="inlineStr">
+      <c r="X12" s="10" t="inlineStr">
         <is>
           <t>366 / 395 C</t>
         </is>
       </c>
-      <c r="X12" s="10" t="inlineStr">
+      <c r="Y12" s="10" t="inlineStr">
         <is>
           <t>45 / 75 C</t>
         </is>
       </c>
-      <c r="Y12" s="10" t="inlineStr">
+      <c r="Z12" s="10" t="inlineStr">
         <is>
           <t>45 / 75 C</t>
         </is>
@@ -20634,30 +20683,35 @@
       </c>
       <c r="T13" s="10" t="inlineStr">
         <is>
+          <t>800 kg/m3</t>
+        </is>
+      </c>
+      <c r="U13" s="10" t="inlineStr">
+        <is>
           <t>737 kg/m3</t>
         </is>
       </c>
-      <c r="U13" s="10" t="inlineStr">
+      <c r="V13" s="10" t="inlineStr">
         <is>
           <t>709 kg/m3</t>
         </is>
       </c>
-      <c r="V13" s="10" t="inlineStr">
+      <c r="W13" s="10" t="inlineStr">
         <is>
           <t>714 kg/m3</t>
         </is>
       </c>
-      <c r="W13" s="10" t="inlineStr">
+      <c r="X13" s="10" t="inlineStr">
         <is>
           <t>761 kg/m3</t>
         </is>
       </c>
-      <c r="X13" s="10" t="inlineStr">
+      <c r="Y13" s="10" t="inlineStr">
         <is>
           <t>990 kg/m3</t>
         </is>
       </c>
-      <c r="Y13" s="10" t="inlineStr">
+      <c r="Z13" s="10" t="inlineStr">
         <is>
           <t>850 kg/m3</t>
         </is>
@@ -20785,6 +20839,11 @@
           <t>TBD (process)</t>
         </is>
       </c>
+      <c r="Z14" s="10" t="inlineStr">
+        <is>
+          <t>TBD (process)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr"/>
@@ -20880,30 +20939,35 @@
       </c>
       <c r="T15" s="10" t="inlineStr">
         <is>
+          <t>Estimated</t>
+        </is>
+      </c>
+      <c r="U15" s="10" t="inlineStr">
+        <is>
           <t>Bubble point (= surface P)</t>
         </is>
       </c>
-      <c r="U15" s="10" t="inlineStr">
+      <c r="V15" s="10" t="inlineStr">
         <is>
           <t>Bubble point (= surface P)</t>
         </is>
       </c>
-      <c r="V15" s="10" t="inlineStr">
+      <c r="W15" s="10" t="inlineStr">
         <is>
           <t>Bubble point (= surface P)</t>
         </is>
       </c>
-      <c r="W15" s="10" t="inlineStr">
+      <c r="X15" s="10" t="inlineStr">
         <is>
           <t>Bubble point (= surface P)</t>
         </is>
       </c>
-      <c r="X15" s="10" t="inlineStr">
+      <c r="Y15" s="10" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
       </c>
-      <c r="Y15" s="10" t="inlineStr">
+      <c r="Z15" s="10" t="inlineStr">
         <is>
           <t>Estimated</t>
         </is>
@@ -21003,30 +21067,35 @@
       </c>
       <c r="T16" s="10" t="inlineStr">
         <is>
+          <t>20.6 / 18.8 m3/h</t>
+        </is>
+      </c>
+      <c r="U16" s="10" t="inlineStr">
+        <is>
           <t>198.3 / 180.3 m3/h</t>
         </is>
       </c>
-      <c r="U16" s="10" t="inlineStr">
+      <c r="V16" s="10" t="inlineStr">
         <is>
           <t>391.0 / 355.4 m3/h</t>
         </is>
       </c>
-      <c r="V16" s="10" t="inlineStr">
+      <c r="W16" s="10" t="inlineStr">
         <is>
           <t>12.2 / 11.1 m3/h</t>
         </is>
       </c>
-      <c r="W16" s="10" t="inlineStr">
+      <c r="X16" s="10" t="inlineStr">
         <is>
           <t>195.6 / 177.8 m3/h</t>
         </is>
       </c>
-      <c r="X16" s="10" t="inlineStr">
+      <c r="Y16" s="10" t="inlineStr">
         <is>
           <t>13.5 / 12.3 m3/h</t>
         </is>
       </c>
-      <c r="Y16" s="10" t="inlineStr">
+      <c r="Z16" s="10" t="inlineStr">
         <is>
           <t>0.6 / 0.6 m3/h</t>
         </is>
@@ -21126,30 +21195,35 @@
       </c>
       <c r="T17" s="10" t="inlineStr">
         <is>
+          <t>0.19 barg</t>
+        </is>
+      </c>
+      <c r="U17" s="10" t="inlineStr">
+        <is>
           <t>1.60 barg</t>
         </is>
       </c>
-      <c r="U17" s="10" t="inlineStr">
+      <c r="V17" s="10" t="inlineStr">
         <is>
           <t>0.98 barg</t>
         </is>
       </c>
-      <c r="V17" s="10" t="inlineStr">
+      <c r="W17" s="10" t="inlineStr">
         <is>
           <t>0.45 barg</t>
         </is>
       </c>
-      <c r="W17" s="10" t="inlineStr">
+      <c r="X17" s="10" t="inlineStr">
         <is>
           <t>-0.55 barg</t>
         </is>
       </c>
-      <c r="X17" s="10" t="inlineStr">
+      <c r="Y17" s="10" t="inlineStr">
         <is>
           <t>-0.02 barg</t>
         </is>
       </c>
-      <c r="Y17" s="10" t="inlineStr">
+      <c r="Z17" s="10" t="inlineStr">
         <is>
           <t>-0.01 barg</t>
         </is>
@@ -21224,7 +21298,7 @@
       </c>
       <c r="O18" s="10" t="inlineStr">
         <is>
-          <t>8.93 barg</t>
+          <t>14.93 barg</t>
         </is>
       </c>
       <c r="P18" s="10" t="inlineStr">
@@ -21249,30 +21323,35 @@
       </c>
       <c r="T18" s="10" t="inlineStr">
         <is>
+          <t>6.19 barg</t>
+        </is>
+      </c>
+      <c r="U18" s="10" t="inlineStr">
+        <is>
           <t>11.60 barg</t>
         </is>
       </c>
-      <c r="U18" s="10" t="inlineStr">
+      <c r="V18" s="10" t="inlineStr">
         <is>
           <t>10.98 barg</t>
         </is>
       </c>
-      <c r="V18" s="10" t="inlineStr">
+      <c r="W18" s="10" t="inlineStr">
         <is>
           <t>8.45 barg</t>
         </is>
       </c>
-      <c r="W18" s="10" t="inlineStr">
+      <c r="X18" s="10" t="inlineStr">
         <is>
           <t>13.45 barg</t>
         </is>
       </c>
-      <c r="X18" s="10" t="inlineStr">
+      <c r="Y18" s="10" t="inlineStr">
         <is>
           <t>4.98 barg</t>
         </is>
       </c>
-      <c r="Y18" s="10" t="inlineStr">
+      <c r="Z18" s="10" t="inlineStr">
         <is>
           <t>4.99 barg</t>
         </is>
@@ -21347,7 +21426,7 @@
       </c>
       <c r="O19" s="10" t="inlineStr">
         <is>
-          <t>8.0 bar / 82 m</t>
+          <t>14.0 bar / 144 m</t>
         </is>
       </c>
       <c r="P19" s="10" t="inlineStr">
@@ -21372,30 +21451,35 @@
       </c>
       <c r="T19" s="10" t="inlineStr">
         <is>
+          <t>6.0 bar / 76 m</t>
+        </is>
+      </c>
+      <c r="U19" s="10" t="inlineStr">
+        <is>
           <t>10.0 bar / 138 m</t>
         </is>
       </c>
-      <c r="U19" s="10" t="inlineStr">
+      <c r="V19" s="10" t="inlineStr">
         <is>
           <t>10.0 bar / 144 m</t>
         </is>
       </c>
-      <c r="V19" s="10" t="inlineStr">
+      <c r="W19" s="10" t="inlineStr">
         <is>
           <t>8.0 bar / 114 m</t>
         </is>
       </c>
-      <c r="W19" s="10" t="inlineStr">
+      <c r="X19" s="10" t="inlineStr">
         <is>
           <t>14.0 bar / 187 m</t>
         </is>
       </c>
-      <c r="X19" s="10" t="inlineStr">
+      <c r="Y19" s="10" t="inlineStr">
         <is>
           <t>5.0 bar / 51 m</t>
         </is>
       </c>
-      <c r="Y19" s="10" t="inlineStr">
+      <c r="Z19" s="10" t="inlineStr">
         <is>
           <t>5.0 bar / 60 m</t>
         </is>
@@ -21495,30 +21579,35 @@
       </c>
       <c r="T20" s="10" t="inlineStr">
         <is>
+          <t>-0.1 m</t>
+        </is>
+      </c>
+      <c r="U20" s="10" t="inlineStr">
+        <is>
           <t>35.7 m</t>
         </is>
       </c>
-      <c r="U20" s="10" t="inlineStr">
+      <c r="V20" s="10" t="inlineStr">
         <is>
           <t>28.1 m</t>
         </is>
       </c>
-      <c r="V20" s="10" t="inlineStr">
+      <c r="W20" s="10" t="inlineStr">
         <is>
           <t>20.0 m</t>
         </is>
       </c>
-      <c r="W20" s="10" t="inlineStr">
+      <c r="X20" s="10" t="inlineStr">
         <is>
           <t>5.2 m</t>
         </is>
       </c>
-      <c r="X20" s="10" t="inlineStr">
+      <c r="Y20" s="10" t="inlineStr">
         <is>
           <t>9.3 m</t>
         </is>
       </c>
-      <c r="Y20" s="10" t="inlineStr">
+      <c r="Z20" s="10" t="inlineStr">
         <is>
           <t>11.4 m</t>
         </is>
@@ -21618,30 +21707,35 @@
       </c>
       <c r="T21" s="10" t="inlineStr">
         <is>
+          <t>0.6 m</t>
+        </is>
+      </c>
+      <c r="U21" s="10" t="inlineStr">
+        <is>
           <t>2.7 m</t>
         </is>
       </c>
-      <c r="U21" s="10" t="inlineStr">
+      <c r="V21" s="10" t="inlineStr">
         <is>
           <t>4.2 m</t>
         </is>
       </c>
-      <c r="V21" s="10" t="inlineStr">
+      <c r="W21" s="10" t="inlineStr">
         <is>
           <t>1.0 m</t>
         </is>
       </c>
-      <c r="W21" s="10" t="inlineStr">
+      <c r="X21" s="10" t="inlineStr">
         <is>
           <t>2.6 m</t>
         </is>
       </c>
-      <c r="X21" s="10" t="inlineStr">
+      <c r="Y21" s="10" t="inlineStr">
         <is>
           <t>1.1 m</t>
         </is>
       </c>
-      <c r="Y21" s="10" t="inlineStr">
+      <c r="Z21" s="10" t="inlineStr">
         <is>
           <t>0.1 m</t>
         </is>
@@ -21741,30 +21835,35 @@
       </c>
       <c r="T22" s="10" t="inlineStr">
         <is>
+          <t>-0.7 m</t>
+        </is>
+      </c>
+      <c r="U22" s="10" t="inlineStr">
+        <is>
           <t>33.0 m</t>
         </is>
       </c>
-      <c r="U22" s="10" t="inlineStr">
+      <c r="V22" s="10" t="inlineStr">
         <is>
           <t>23.9 m</t>
         </is>
       </c>
-      <c r="V22" s="10" t="inlineStr">
+      <c r="W22" s="10" t="inlineStr">
         <is>
           <t>19.0 m</t>
         </is>
       </c>
-      <c r="W22" s="10" t="inlineStr">
+      <c r="X22" s="10" t="inlineStr">
         <is>
           <t>2.6 m</t>
         </is>
       </c>
-      <c r="X22" s="10" t="inlineStr">
+      <c r="Y22" s="10" t="inlineStr">
         <is>
           <t>8.1 m</t>
         </is>
       </c>
-      <c r="Y22" s="10" t="inlineStr">
+      <c r="Z22" s="10" t="inlineStr">
         <is>
           <t>11.3 m</t>
         </is>
@@ -21839,7 +21938,7 @@
       </c>
       <c r="O23" s="10" t="inlineStr">
         <is>
-          <t>8.2 kW</t>
+          <t>14.3 kW</t>
         </is>
       </c>
       <c r="P23" s="10" t="inlineStr">
@@ -21864,30 +21963,35 @@
       </c>
       <c r="T23" s="10" t="inlineStr">
         <is>
+          <t>3.4 kW</t>
+        </is>
+      </c>
+      <c r="U23" s="10" t="inlineStr">
+        <is>
           <t>55.1 kW</t>
         </is>
       </c>
-      <c r="U23" s="10" t="inlineStr">
+      <c r="V23" s="10" t="inlineStr">
         <is>
           <t>108.6 kW</t>
         </is>
       </c>
-      <c r="V23" s="10" t="inlineStr">
+      <c r="W23" s="10" t="inlineStr">
         <is>
           <t>2.7 kW</t>
         </is>
       </c>
-      <c r="W23" s="10" t="inlineStr">
+      <c r="X23" s="10" t="inlineStr">
         <is>
           <t>76.1 kW</t>
         </is>
       </c>
-      <c r="X23" s="10" t="inlineStr">
+      <c r="Y23" s="10" t="inlineStr">
         <is>
           <t>1.9 kW</t>
         </is>
       </c>
-      <c r="Y23" s="10" t="inlineStr">
+      <c r="Z23" s="10" t="inlineStr">
         <is>
           <t>0.1 kW</t>
         </is>
@@ -21987,30 +22091,35 @@
       </c>
       <c r="T24" s="10" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U24" s="10" t="inlineStr">
+        <is>
           <t>Sour (H2S) / naphthenic</t>
         </is>
       </c>
-      <c r="U24" s="10" t="inlineStr">
+      <c r="V24" s="10" t="inlineStr">
         <is>
           <t>Sour (H2S) / naphthenic</t>
         </is>
       </c>
-      <c r="V24" s="10" t="inlineStr">
+      <c r="W24" s="10" t="inlineStr">
         <is>
           <t>Sour (H2S) / naphthenic</t>
         </is>
       </c>
-      <c r="W24" s="10" t="inlineStr">
+      <c r="X24" s="10" t="inlineStr">
         <is>
           <t>Sour (H2S) / naphthenic</t>
         </is>
       </c>
-      <c r="X24" s="10" t="inlineStr">
+      <c r="Y24" s="10" t="inlineStr">
         <is>
           <t>Sour</t>
         </is>
       </c>
-      <c r="Y24" s="10" t="inlineStr">
+      <c r="Z24" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -22046,6 +22155,7 @@
       <c r="W25" s="8" t="n"/>
       <c r="X25" s="8" t="n"/>
       <c r="Y25" s="8" t="n"/>
+      <c r="Z25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr"/>
@@ -22151,20 +22261,25 @@
       </c>
       <c r="V26" s="10" t="inlineStr">
         <is>
+          <t>1780 rpm</t>
+        </is>
+      </c>
+      <c r="W26" s="10" t="inlineStr">
+        <is>
           <t>3560 rpm</t>
         </is>
       </c>
-      <c r="W26" s="10" t="inlineStr">
+      <c r="X26" s="10" t="inlineStr">
         <is>
           <t>1780 rpm</t>
         </is>
       </c>
-      <c r="X26" s="10" t="inlineStr">
+      <c r="Y26" s="10" t="inlineStr">
         <is>
           <t>3560 rpm</t>
         </is>
       </c>
-      <c r="Y26" s="10" t="inlineStr">
+      <c r="Z26" s="10" t="inlineStr">
         <is>
           <t>3560 rpm</t>
         </is>
@@ -22279,15 +22394,20 @@
       </c>
       <c r="W27" s="10" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X27" s="10" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="X27" s="10" t="inlineStr">
+      <c r="Y27" s="10" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="Y27" s="10" t="inlineStr">
+      <c r="Z27" s="10" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -22387,30 +22507,35 @@
       </c>
       <c r="T28" s="10" t="inlineStr">
         <is>
+          <t>60 %</t>
+        </is>
+      </c>
+      <c r="U28" s="10" t="inlineStr">
+        <is>
           <t>68 %</t>
         </is>
       </c>
-      <c r="U28" s="10" t="inlineStr">
+      <c r="V28" s="10" t="inlineStr">
         <is>
           <t>70 %</t>
         </is>
       </c>
-      <c r="V28" s="10" t="inlineStr">
+      <c r="W28" s="10" t="inlineStr">
         <is>
           <t>58 %</t>
         </is>
       </c>
-      <c r="W28" s="10" t="inlineStr">
+      <c r="X28" s="10" t="inlineStr">
         <is>
           <t>68 %</t>
         </is>
       </c>
-      <c r="X28" s="10" t="inlineStr">
+      <c r="Y28" s="10" t="inlineStr">
         <is>
           <t>58 %</t>
         </is>
       </c>
-      <c r="Y28" s="10" t="inlineStr">
+      <c r="Z28" s="10" t="inlineStr">
         <is>
           <t>55 %</t>
         </is>
@@ -22485,7 +22610,7 @@
       </c>
       <c r="O29" s="10" t="inlineStr">
         <is>
-          <t>13.2 kW</t>
+          <t>23.1 kW</t>
         </is>
       </c>
       <c r="P29" s="10" t="inlineStr">
@@ -22510,30 +22635,35 @@
       </c>
       <c r="T29" s="10" t="inlineStr">
         <is>
+          <t>5.7 kW</t>
+        </is>
+      </c>
+      <c r="U29" s="10" t="inlineStr">
+        <is>
           <t>81.3 kW</t>
         </is>
       </c>
-      <c r="U29" s="10" t="inlineStr">
+      <c r="V29" s="10" t="inlineStr">
         <is>
           <t>154.8 kW</t>
         </is>
       </c>
-      <c r="V29" s="10" t="inlineStr">
+      <c r="W29" s="10" t="inlineStr">
         <is>
           <t>4.7 kW</t>
         </is>
       </c>
-      <c r="W29" s="10" t="inlineStr">
+      <c r="X29" s="10" t="inlineStr">
         <is>
           <t>112.3 kW</t>
         </is>
       </c>
-      <c r="X29" s="10" t="inlineStr">
+      <c r="Y29" s="10" t="inlineStr">
         <is>
           <t>3.2 kW</t>
         </is>
       </c>
-      <c r="Y29" s="10" t="inlineStr">
+      <c r="Z29" s="10" t="inlineStr">
         <is>
           <t>0.2 kW</t>
         </is>
@@ -22608,14 +22738,14 @@
       </c>
       <c r="O30" s="10" t="inlineStr">
         <is>
+          <t>30 kW</t>
+        </is>
+      </c>
+      <c r="P30" s="10" t="inlineStr">
+        <is>
           <t>18.5 kW</t>
         </is>
       </c>
-      <c r="P30" s="10" t="inlineStr">
-        <is>
-          <t>18.5 kW</t>
-        </is>
-      </c>
       <c r="Q30" s="10" t="inlineStr">
         <is>
           <t>55 kW</t>
@@ -22633,30 +22763,35 @@
       </c>
       <c r="T30" s="10" t="inlineStr">
         <is>
+          <t>7.5 kW</t>
+        </is>
+      </c>
+      <c r="U30" s="10" t="inlineStr">
+        <is>
           <t>110 kW</t>
         </is>
       </c>
-      <c r="U30" s="10" t="inlineStr">
+      <c r="V30" s="10" t="inlineStr">
         <is>
           <t>200 kW</t>
         </is>
       </c>
-      <c r="V30" s="10" t="inlineStr">
+      <c r="W30" s="10" t="inlineStr">
         <is>
           <t>5.5 kW</t>
         </is>
       </c>
-      <c r="W30" s="10" t="inlineStr">
+      <c r="X30" s="10" t="inlineStr">
         <is>
           <t>132 kW</t>
         </is>
       </c>
-      <c r="X30" s="10" t="inlineStr">
+      <c r="Y30" s="10" t="inlineStr">
         <is>
           <t>3.7 kW</t>
         </is>
       </c>
-      <c r="Y30" s="10" t="inlineStr">
+      <c r="Z30" s="10" t="inlineStr">
         <is>
           <t>0.75 kW</t>
         </is>
@@ -22761,25 +22896,30 @@
       </c>
       <c r="U31" s="10" t="inlineStr">
         <is>
+          <t>480 V, 3 ph, 60 Hz</t>
+        </is>
+      </c>
+      <c r="V31" s="10" t="inlineStr">
+        <is>
           <t>4.16 kV, 3 ph, 60 Hz</t>
         </is>
       </c>
-      <c r="V31" s="10" t="inlineStr">
+      <c r="W31" s="10" t="inlineStr">
         <is>
           <t>480 V, 3 ph, 60 Hz</t>
         </is>
       </c>
-      <c r="W31" s="10" t="inlineStr">
+      <c r="X31" s="10" t="inlineStr">
         <is>
           <t>480 V, 3 ph, 60 Hz</t>
         </is>
       </c>
-      <c r="X31" s="10" t="inlineStr">
+      <c r="Y31" s="10" t="inlineStr">
         <is>
           <t>480 V, 3 ph, 60 Hz</t>
         </is>
       </c>
-      <c r="Y31" s="10" t="inlineStr">
+      <c r="Z31" s="10" t="inlineStr">
         <is>
           <t>480 V, 3 ph, 60 Hz</t>
         </is>
@@ -22907,6 +23047,11 @@
           <t>TEFC, Class I Div 2 Gr D / Zone 2 IIA T3</t>
         </is>
       </c>
+      <c r="Z32" s="10" t="inlineStr">
+        <is>
+          <t>TEFC, Class I Div 2 Gr D / Zone 2 IIA T3</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr"/>
@@ -23002,30 +23147,35 @@
       </c>
       <c r="T33" s="10" t="inlineStr">
         <is>
+          <t>3" / 2" 300# RF (vendor)</t>
+        </is>
+      </c>
+      <c r="U33" s="10" t="inlineStr">
+        <is>
           <t>8" / 6" 300# RF (vendor)</t>
         </is>
       </c>
-      <c r="U33" s="10" t="inlineStr">
+      <c r="V33" s="10" t="inlineStr">
         <is>
           <t>10" / 8" 300# RF (vendor)</t>
         </is>
       </c>
-      <c r="V33" s="10" t="inlineStr">
+      <c r="W33" s="10" t="inlineStr">
         <is>
           <t>2" / 2" 300# RF (vendor)</t>
         </is>
       </c>
-      <c r="W33" s="10" t="inlineStr">
+      <c r="X33" s="10" t="inlineStr">
         <is>
           <t>8" / 6" 300# RF (vendor)</t>
         </is>
       </c>
-      <c r="X33" s="10" t="inlineStr">
+      <c r="Y33" s="10" t="inlineStr">
         <is>
           <t>2" / 2" 300# RF (vendor)</t>
         </is>
       </c>
-      <c r="Y33" s="10" t="inlineStr">
+      <c r="Z33" s="10" t="inlineStr">
         <is>
           <t>2" / 2" 300# RF (vendor)</t>
         </is>
@@ -23153,6 +23303,11 @@
           <t>40 barg (incl. shut-off, TBD)</t>
         </is>
       </c>
+      <c r="Z34" s="10" t="inlineStr">
+        <is>
+          <t>40 barg (incl. shut-off, TBD)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr"/>
@@ -23253,25 +23408,30 @@
       </c>
       <c r="U35" s="10" t="inlineStr">
         <is>
+          <t>S-6 (CS/12Cr)</t>
+        </is>
+      </c>
+      <c r="V35" s="10" t="inlineStr">
+        <is>
           <t>A-8 (316)</t>
         </is>
       </c>
-      <c r="V35" s="10" t="inlineStr">
+      <c r="W35" s="10" t="inlineStr">
         <is>
           <t>A-8 (316)</t>
         </is>
       </c>
-      <c r="W35" s="10" t="inlineStr">
+      <c r="X35" s="10" t="inlineStr">
         <is>
           <t>A-8 (316)</t>
         </is>
       </c>
-      <c r="X35" s="10" t="inlineStr">
+      <c r="Y35" s="10" t="inlineStr">
         <is>
           <t>S-6 (CS/12Cr)</t>
         </is>
       </c>
-      <c r="Y35" s="10" t="inlineStr">
+      <c r="Z35" s="10" t="inlineStr">
         <is>
           <t>S-6 (CS/12Cr)</t>
         </is>
@@ -23376,25 +23536,30 @@
       </c>
       <c r="U36" s="10" t="inlineStr">
         <is>
+          <t>API 682 Plan 11/52, API 682 Cat 2, Arr. 1</t>
+        </is>
+      </c>
+      <c r="V36" s="10" t="inlineStr">
+        <is>
           <t>API 682 Plan 53B, API 682 Cat 2, Arr. 2</t>
         </is>
       </c>
-      <c r="V36" s="10" t="inlineStr">
+      <c r="W36" s="10" t="inlineStr">
         <is>
           <t>API 682 Plan 53B, API 682 Cat 2, Arr. 2</t>
         </is>
       </c>
-      <c r="W36" s="10" t="inlineStr">
+      <c r="X36" s="10" t="inlineStr">
         <is>
           <t>API 682 Plan 53B, API 682 Cat 2, Arr. 2</t>
         </is>
       </c>
-      <c r="X36" s="10" t="inlineStr">
+      <c r="Y36" s="10" t="inlineStr">
         <is>
           <t>API 682 Plan 11/52, API 682 Cat 2, Arr. 1</t>
         </is>
       </c>
-      <c r="Y36" s="10" t="inlineStr">
+      <c r="Z36" s="10" t="inlineStr">
         <is>
           <t>API 682 Plan 11/52, API 682 Cat 2, Arr. 1</t>
         </is>
@@ -23522,6 +23687,11 @@
           <t>Rolling / ring oil</t>
         </is>
       </c>
+      <c r="Z37" s="10" t="inlineStr">
+        <is>
+          <t>Rolling / ring oil</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr"/>
@@ -23645,6 +23815,11 @@
           <t>Flexible disc spacer / API 610 grouted</t>
         </is>
       </c>
+      <c r="Z38" s="10" t="inlineStr">
+        <is>
+          <t>Flexible disc spacer / API 610 grouted</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr"/>
@@ -23768,6 +23943,11 @@
           <t>Vendor (min. flow bypass if &lt; 30 % rated)</t>
         </is>
       </c>
+      <c r="Z39" s="10" t="inlineStr">
+        <is>
+          <t>Vendor (min. flow bypass if &lt; 30 % rated)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr"/>
@@ -23838,14 +24018,14 @@
       </c>
       <c r="O40" s="10" t="inlineStr">
         <is>
+          <t>0.7 t each</t>
+        </is>
+      </c>
+      <c r="P40" s="10" t="inlineStr">
+        <is>
           <t>0.5 t each</t>
         </is>
       </c>
-      <c r="P40" s="10" t="inlineStr">
-        <is>
-          <t>0.5 t each</t>
-        </is>
-      </c>
       <c r="Q40" s="10" t="inlineStr">
         <is>
           <t>1.0 t each</t>
@@ -23863,30 +24043,35 @@
       </c>
       <c r="T40" s="10" t="inlineStr">
         <is>
+          <t>0.4 t each</t>
+        </is>
+      </c>
+      <c r="U40" s="10" t="inlineStr">
+        <is>
           <t>2.7 t each</t>
         </is>
       </c>
-      <c r="U40" s="10" t="inlineStr">
+      <c r="V40" s="10" t="inlineStr">
         <is>
           <t>4.2 t each</t>
         </is>
       </c>
-      <c r="V40" s="10" t="inlineStr">
+      <c r="W40" s="10" t="inlineStr">
         <is>
           <t>0.9 t each</t>
         </is>
       </c>
-      <c r="W40" s="10" t="inlineStr">
+      <c r="X40" s="10" t="inlineStr">
         <is>
           <t>3.0 t each</t>
         </is>
       </c>
-      <c r="X40" s="10" t="inlineStr">
+      <c r="Y40" s="10" t="inlineStr">
         <is>
           <t>0.3 t each</t>
         </is>
       </c>
-      <c r="Y40" s="10" t="inlineStr">
+      <c r="Z40" s="10" t="inlineStr">
         <is>
           <t>0.3 t each</t>
         </is>
@@ -23903,7 +24088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -23920,6 +24105,9 @@
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -23941,6 +24129,9 @@
       <c r="L1" t="inlineStr"/>
       <c r="M1" t="inlineStr"/>
       <c r="N1" t="inlineStr"/>
+      <c r="O1" t="inlineStr"/>
+      <c r="P1" t="inlineStr"/>
+      <c r="Q1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -24011,6 +24202,21 @@
       <c r="N2" s="5" t="inlineStr">
         <is>
           <t>PSV-2002</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>PSV-1011</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>PSV-2003</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>TSV-typ</t>
         </is>
       </c>
     </row>
@@ -24033,6 +24239,9 @@
       <c r="L3" s="8" t="n"/>
       <c r="M3" s="8" t="n"/>
       <c r="N3" s="8" t="n"/>
+      <c r="O3" s="8" t="n"/>
+      <c r="P3" s="8" t="n"/>
+      <c r="Q3" s="8" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr"/>
@@ -24101,6 +24310,21 @@
           <t>PSV-2002 / 1</t>
         </is>
       </c>
+      <c r="O4" s="10" t="inlineStr">
+        <is>
+          <t>PSV-1011 / 1</t>
+        </is>
+      </c>
+      <c r="P4" s="10" t="inlineStr">
+        <is>
+          <t>PSV-2003 / 1</t>
+        </is>
+      </c>
+      <c r="Q4" s="10" t="inlineStr">
+        <is>
+          <t>TSV-typ / 1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr"/>
@@ -24169,6 +24393,21 @@
           <t>D-201</t>
         </is>
       </c>
+      <c r="O5" s="10" t="inlineStr">
+        <is>
+          <t>E-113 (steam side)</t>
+        </is>
+      </c>
+      <c r="P5" s="10" t="inlineStr">
+        <is>
+          <t>E-201 (steam side)</t>
+        </is>
+      </c>
+      <c r="Q5" s="10" t="inlineStr">
+        <is>
+          <t>CW sides E-115, E-202..E-204</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr"/>
@@ -24237,6 +24476,21 @@
           <t>Fire</t>
         </is>
       </c>
+      <c r="O6" s="10" t="inlineStr">
+        <is>
+          <t>Blocked MP steam outlet (max. generation)</t>
+        </is>
+      </c>
+      <c r="P6" s="10" t="inlineStr">
+        <is>
+          <t>Blocked LP steam outlet (max. generation)</t>
+        </is>
+      </c>
+      <c r="Q6" s="10" t="inlineStr">
+        <is>
+          <t>Thermal expansion (blocked-in CW)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr"/>
@@ -24305,6 +24559,21 @@
           <t>Spring-loaded, full-nozzle, high-lift</t>
         </is>
       </c>
+      <c r="O7" s="10" t="inlineStr">
+        <is>
+          <t>Spring-loaded, full-nozzle, high-lift</t>
+        </is>
+      </c>
+      <c r="P7" s="10" t="inlineStr">
+        <is>
+          <t>Spring-loaded, full-nozzle, high-lift</t>
+        </is>
+      </c>
+      <c r="Q7" s="10" t="inlineStr">
+        <is>
+          <t>Spring-loaded, full-nozzle, high-lift</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr"/>
@@ -24373,6 +24642,21 @@
           <t>Balanced bellows</t>
         </is>
       </c>
+      <c r="O8" s="10" t="inlineStr">
+        <is>
+          <t>Conventional</t>
+        </is>
+      </c>
+      <c r="P8" s="10" t="inlineStr">
+        <is>
+          <t>Conventional</t>
+        </is>
+      </c>
+      <c r="Q8" s="10" t="inlineStr">
+        <is>
+          <t>Conventional</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr"/>
@@ -24441,6 +24725,21 @@
           <t>Flare</t>
         </is>
       </c>
+      <c r="O9" s="10" t="inlineStr">
+        <is>
+          <t>Atmosphere (safe location)</t>
+        </is>
+      </c>
+      <c r="P9" s="10" t="inlineStr">
+        <is>
+          <t>Atmosphere (safe location)</t>
+        </is>
+      </c>
+      <c r="Q9" s="10" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr"/>
@@ -24509,6 +24808,21 @@
           <t>3K4  (inlet x orifice x outlet)</t>
         </is>
       </c>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>3L4  (inlet x orifice x outlet)</t>
+        </is>
+      </c>
+      <c r="P10" s="10" t="inlineStr">
+        <is>
+          <t>3K4  (inlet x orifice x outlet)</t>
+        </is>
+      </c>
+      <c r="Q10" s="10" t="inlineStr">
+        <is>
+          <t>1D2  (inlet x orifice x outlet)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr"/>
@@ -24577,6 +24891,21 @@
           <t>3" 150# RF</t>
         </is>
       </c>
+      <c r="O11" s="10" t="inlineStr">
+        <is>
+          <t>3" 300# RF</t>
+        </is>
+      </c>
+      <c r="P11" s="10" t="inlineStr">
+        <is>
+          <t>3" 150# RF</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>1" 150# RF</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr"/>
@@ -24643,6 +24972,21 @@
       <c r="N12" s="10" t="inlineStr">
         <is>
           <t>4" 150# RF</t>
+        </is>
+      </c>
+      <c r="O12" s="10" t="inlineStr">
+        <is>
+          <t>4" 150# RF</t>
+        </is>
+      </c>
+      <c r="P12" s="10" t="inlineStr">
+        <is>
+          <t>4" 150# RF</t>
+        </is>
+      </c>
+      <c r="Q12" s="10" t="inlineStr">
+        <is>
+          <t>2" 150# RF</t>
         </is>
       </c>
     </row>
@@ -24665,6 +25009,9 @@
       <c r="L13" s="8" t="n"/>
       <c r="M13" s="8" t="n"/>
       <c r="N13" s="8" t="n"/>
+      <c r="O13" s="8" t="n"/>
+      <c r="P13" s="8" t="n"/>
+      <c r="Q13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr"/>
@@ -24733,6 +25080,21 @@
           <t>Hydrocarbon vapour</t>
         </is>
       </c>
+      <c r="O14" s="10" t="inlineStr">
+        <is>
+          <t>Steam / vapour</t>
+        </is>
+      </c>
+      <c r="P14" s="10" t="inlineStr">
+        <is>
+          <t>Steam / vapour</t>
+        </is>
+      </c>
+      <c r="Q14" s="10" t="inlineStr">
+        <is>
+          <t>Steam / vapour</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr"/>
@@ -24801,6 +25163,21 @@
           <t>6,324 kg/h</t>
         </is>
       </c>
+      <c r="O15" s="10" t="inlineStr">
+        <is>
+          <t>8,833 kg/h</t>
+        </is>
+      </c>
+      <c r="P15" s="10" t="inlineStr">
+        <is>
+          <t>3,054 kg/h</t>
+        </is>
+      </c>
+      <c r="Q15" s="10" t="inlineStr">
+        <is>
+          <t>50 kg/h</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr"/>
@@ -24869,6 +25246,21 @@
           <t>100.0</t>
         </is>
       </c>
+      <c r="O16" s="10" t="inlineStr">
+        <is>
+          <t>18.0</t>
+        </is>
+      </c>
+      <c r="P16" s="10" t="inlineStr">
+        <is>
+          <t>18.0</t>
+        </is>
+      </c>
+      <c r="Q16" s="10" t="inlineStr">
+        <is>
+          <t>18.0</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr"/>
@@ -24937,6 +25329,21 @@
           <t>120 C</t>
         </is>
       </c>
+      <c r="O17" s="10" t="inlineStr">
+        <is>
+          <t>186 C</t>
+        </is>
+      </c>
+      <c r="P17" s="10" t="inlineStr">
+        <is>
+          <t>148 C</t>
+        </is>
+      </c>
+      <c r="Q17" s="10" t="inlineStr">
+        <is>
+          <t>60 C</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr"/>
@@ -25005,6 +25412,21 @@
           <t>1.10 / 1.0</t>
         </is>
       </c>
+      <c r="O18" s="10" t="inlineStr">
+        <is>
+          <t>1.10 / 1.0</t>
+        </is>
+      </c>
+      <c r="P18" s="10" t="inlineStr">
+        <is>
+          <t>1.10 / 1.0</t>
+        </is>
+      </c>
+      <c r="Q18" s="10" t="inlineStr">
+        <is>
+          <t>1.10 / 1.0</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr"/>
@@ -25073,6 +25495,21 @@
           <t>3.5 barg</t>
         </is>
       </c>
+      <c r="O19" s="10" t="inlineStr">
+        <is>
+          <t>12.0 barg</t>
+        </is>
+      </c>
+      <c r="P19" s="10" t="inlineStr">
+        <is>
+          <t>5.0 barg</t>
+        </is>
+      </c>
+      <c r="Q19" s="10" t="inlineStr">
+        <is>
+          <t>7.0 barg</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr"/>
@@ -25141,6 +25578,21 @@
           <t>21 % (fire)</t>
         </is>
       </c>
+      <c r="O20" s="10" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="P20" s="10" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
+      <c r="Q20" s="10" t="inlineStr">
+        <is>
+          <t>10 %</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr"/>
@@ -25209,6 +25661,21 @@
           <t>0.5 barg superimposed (var.) + 10 % built-up</t>
         </is>
       </c>
+      <c r="O21" s="10" t="inlineStr">
+        <is>
+          <t>atm</t>
+        </is>
+      </c>
+      <c r="P21" s="10" t="inlineStr">
+        <is>
+          <t>atm</t>
+        </is>
+      </c>
+      <c r="Q21" s="10" t="inlineStr">
+        <is>
+          <t>atm</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr"/>
@@ -25277,6 +25744,21 @@
           <t>0.975 / 1.0 / 1.0</t>
         </is>
       </c>
+      <c r="O22" s="10" t="inlineStr">
+        <is>
+          <t>0.975 / 1.0 / 1.0</t>
+        </is>
+      </c>
+      <c r="P22" s="10" t="inlineStr">
+        <is>
+          <t>0.975 / 1.0 / 1.0</t>
+        </is>
+      </c>
+      <c r="Q22" s="10" t="inlineStr">
+        <is>
+          <t>0.975 / 1.0 / 1.0</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr"/>
@@ -25345,6 +25827,21 @@
           <t>1,066 mm2</t>
         </is>
       </c>
+      <c r="O23" s="10" t="inlineStr">
+        <is>
+          <t>1,298 mm2</t>
+        </is>
+      </c>
+      <c r="P23" s="10" t="inlineStr">
+        <is>
+          <t>938 mm2</t>
+        </is>
+      </c>
+      <c r="Q23" s="10" t="inlineStr">
+        <is>
+          <t>10 mm2</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr"/>
@@ -25413,6 +25910,21 @@
           <t>K / 1,186 mm2 each</t>
         </is>
       </c>
+      <c r="O24" s="10" t="inlineStr">
+        <is>
+          <t>L / 1,841 mm2 each</t>
+        </is>
+      </c>
+      <c r="P24" s="10" t="inlineStr">
+        <is>
+          <t>K / 1,186 mm2 each</t>
+        </is>
+      </c>
+      <c r="Q24" s="10" t="inlineStr">
+        <is>
+          <t>D / 71 mm2 each</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr"/>
@@ -25481,6 +25993,21 @@
           <t>90 %</t>
         </is>
       </c>
+      <c r="O25" s="10" t="inlineStr">
+        <is>
+          <t>70 %</t>
+        </is>
+      </c>
+      <c r="P25" s="10" t="inlineStr">
+        <is>
+          <t>79 %</t>
+        </is>
+      </c>
+      <c r="Q25" s="10" t="inlineStr">
+        <is>
+          <t>14 %</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr"/>
@@ -25545,6 +26072,21 @@
         </is>
       </c>
       <c r="N26" s="10" t="inlineStr">
+        <is>
+          <t>&lt; 3 % of set (API 520-II)</t>
+        </is>
+      </c>
+      <c r="O26" s="10" t="inlineStr">
+        <is>
+          <t>&lt; 3 % of set (API 520-II)</t>
+        </is>
+      </c>
+      <c r="P26" s="10" t="inlineStr">
+        <is>
+          <t>&lt; 3 % of set (API 520-II)</t>
+        </is>
+      </c>
+      <c r="Q26" s="10" t="inlineStr">
         <is>
           <t>&lt; 3 % of set (API 520-II)</t>
         </is>
@@ -25569,6 +26111,9 @@
       <c r="L27" s="8" t="n"/>
       <c r="M27" s="8" t="n"/>
       <c r="N27" s="8" t="n"/>
+      <c r="O27" s="8" t="n"/>
+      <c r="P27" s="8" t="n"/>
+      <c r="Q27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr"/>
@@ -25637,6 +26182,21 @@
           <t>A216 WCC</t>
         </is>
       </c>
+      <c r="O28" s="10" t="inlineStr">
+        <is>
+          <t>A216 WCC</t>
+        </is>
+      </c>
+      <c r="P28" s="10" t="inlineStr">
+        <is>
+          <t>A216 WCC</t>
+        </is>
+      </c>
+      <c r="Q28" s="10" t="inlineStr">
+        <is>
+          <t>A216 WCC</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr"/>
@@ -25705,6 +26265,21 @@
           <t>316 SS</t>
         </is>
       </c>
+      <c r="O29" s="10" t="inlineStr">
+        <is>
+          <t>316 SS</t>
+        </is>
+      </c>
+      <c r="P29" s="10" t="inlineStr">
+        <is>
+          <t>316 SS</t>
+        </is>
+      </c>
+      <c r="Q29" s="10" t="inlineStr">
+        <is>
+          <t>316 SS</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr"/>
@@ -25773,6 +26348,21 @@
           <t>CS, aluminised (W &lt; 230 C) / tungsten (&gt; 230 C)</t>
         </is>
       </c>
+      <c r="O30" s="10" t="inlineStr">
+        <is>
+          <t>CS, aluminised (W &lt; 230 C) / tungsten (&gt; 230 C)</t>
+        </is>
+      </c>
+      <c r="P30" s="10" t="inlineStr">
+        <is>
+          <t>CS, aluminised (W &lt; 230 C) / tungsten (&gt; 230 C)</t>
+        </is>
+      </c>
+      <c r="Q30" s="10" t="inlineStr">
+        <is>
+          <t>CS, aluminised (W &lt; 230 C) / tungsten (&gt; 230 C)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr"/>
@@ -25841,6 +26431,21 @@
           <t>Inconel 625</t>
         </is>
       </c>
+      <c r="O31" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P31" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q31" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr"/>
@@ -25909,6 +26514,21 @@
           <t>316 SS (Stellited seats)</t>
         </is>
       </c>
+      <c r="O32" s="10" t="inlineStr">
+        <is>
+          <t>316 SS (Stellited seats)</t>
+        </is>
+      </c>
+      <c r="P32" s="10" t="inlineStr">
+        <is>
+          <t>316 SS (Stellited seats)</t>
+        </is>
+      </c>
+      <c r="Q32" s="10" t="inlineStr">
+        <is>
+          <t>316 SS (Stellited seats)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr"/>
@@ -25977,6 +26597,21 @@
           <t>No / Yes</t>
         </is>
       </c>
+      <c r="O33" s="10" t="inlineStr">
+        <is>
+          <t>No / Yes</t>
+        </is>
+      </c>
+      <c r="P33" s="10" t="inlineStr">
+        <is>
+          <t>No / Yes</t>
+        </is>
+      </c>
+      <c r="Q33" s="10" t="inlineStr">
+        <is>
+          <t>No / Yes</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr"/>
@@ -26045,6 +26680,21 @@
           <t>MR0103 (sour)</t>
         </is>
       </c>
+      <c r="O34" s="10" t="inlineStr">
+        <is>
+          <t>MR0103 (sour)</t>
+        </is>
+      </c>
+      <c r="P34" s="10" t="inlineStr">
+        <is>
+          <t>MR0103 (sour)</t>
+        </is>
+      </c>
+      <c r="Q34" s="10" t="inlineStr">
+        <is>
+          <t>MR0103 (sour)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr"/>
@@ -26109,6 +26759,21 @@
         </is>
       </c>
       <c r="N35" s="10" t="inlineStr">
+        <is>
+          <t>ASME VIII-1 UG-125..137, API 520/521/526/527</t>
+        </is>
+      </c>
+      <c r="O35" s="10" t="inlineStr">
+        <is>
+          <t>ASME VIII-1 UG-125..137, API 520/521/526/527</t>
+        </is>
+      </c>
+      <c r="P35" s="10" t="inlineStr">
+        <is>
+          <t>ASME VIII-1 UG-125..137, API 520/521/526/527</t>
+        </is>
+      </c>
+      <c r="Q35" s="10" t="inlineStr">
         <is>
           <t>ASME VIII-1 UG-125..137, API 520/521/526/527</t>
         </is>

</xml_diff>